<commit_message>
Fixed spacing on homepage
</commit_message>
<xml_diff>
--- a/Kabir NEA planner.xlsx
+++ b/Kabir NEA planner.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://swgs-my.sharepoint.com/personal/20kxm_swgs_wilts_sch_uk/Documents/Computer Science/NEA-Quotebook/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="3" documentId="8_{2F616C2B-A507-5E49-B12E-1DC6899D8079}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F866D1A7-0071-44BC-A1F7-93096AED238B}"/>
+  <xr:revisionPtr revIDLastSave="8" documentId="8_{2F616C2B-A507-5E49-B12E-1DC6899D8079}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DE33FDFD-49FE-468E-82AA-576C78D016E9}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="65">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="82" uniqueCount="69">
   <si>
     <t>A-Level Computer Science - Programming Project Planner</t>
   </si>
@@ -228,6 +228,18 @@
   </si>
   <si>
     <t>In Progress</t>
+  </si>
+  <si>
+    <t>Complete</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Research and mood boards of existing products completed. </t>
+  </si>
+  <si>
+    <t>Design outlined and goals set</t>
+  </si>
+  <si>
+    <t>Git set up, ui outlined in bootstrap. No backend started yet</t>
   </si>
 </sst>
 </file>
@@ -389,6 +401,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -746,9 +762,11 @@
       <c r="D5" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="E5" s="5"/>
+      <c r="E5" s="5" t="s">
+        <v>66</v>
+      </c>
       <c r="F5" s="6" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="G5" s="5"/>
     </row>
@@ -765,9 +783,11 @@
       <c r="D6" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="E6" s="9"/>
+      <c r="E6" s="9" t="s">
+        <v>67</v>
+      </c>
       <c r="F6" s="10" t="s">
-        <v>13</v>
+        <v>64</v>
       </c>
       <c r="G6" s="9"/>
     </row>
@@ -822,7 +842,9 @@
       <c r="D9" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="E9" s="5"/>
+      <c r="E9" s="5" t="s">
+        <v>68</v>
+      </c>
       <c r="F9" s="6" t="s">
         <v>64</v>
       </c>
@@ -1158,20 +1180,20 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <ReferenceId xmlns="37a59701-210d-47b6-ae01-fca6546d58ce" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
   <Edit>DocumentLibraryForm</Edit>
   <New>DocumentLibraryForm</New>
 </FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <ReferenceId xmlns="37a59701-210d-47b6-ae01-fca6546d58ce" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1193,6 +1215,14 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{569F84B1-45EB-4542-821C-A957A49172A3}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0466E9FC-0FC4-4755-B69E-E404DE005AA0}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
@@ -1200,12 +1230,4 @@
     <ds:schemaRef ds:uri="37a59701-210d-47b6-ae01-fca6546d58ce"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{569F84B1-45EB-4542-821C-A957A49172A3}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Started overhaul of quote ui
</commit_message>
<xml_diff>
--- a/Kabir NEA planner.xlsx
+++ b/Kabir NEA planner.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://swgs-my.sharepoint.com/personal/20kxm_swgs_wilts_sch_uk/Documents/Computer Science/NEA-Quotebook/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="8" documentId="8_{2F616C2B-A507-5E49-B12E-1DC6899D8079}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DE33FDFD-49FE-468E-82AA-576C78D016E9}"/>
+  <xr:revisionPtr revIDLastSave="10" documentId="8_{2F616C2B-A507-5E49-B12E-1DC6899D8079}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A329382C-3EAB-41A3-BAB0-C166FC4DFC19}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="82" uniqueCount="69">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="83" uniqueCount="70">
   <si>
     <t>A-Level Computer Science - Programming Project Planner</t>
   </si>
@@ -240,6 +240,9 @@
   </si>
   <si>
     <t>Git set up, ui outlined in bootstrap. No backend started yet</t>
+  </si>
+  <si>
+    <t>Hand drawn the ui elements, and am about 60% through outlining in HTML and bootstrap</t>
   </si>
 </sst>
 </file>
@@ -823,9 +826,11 @@
       <c r="D8" s="8" t="s">
         <v>23</v>
       </c>
-      <c r="E8" s="9"/>
+      <c r="E8" s="9" t="s">
+        <v>69</v>
+      </c>
       <c r="F8" s="10" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="G8" s="9"/>
     </row>
@@ -1036,6 +1041,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100A74177071F0F0C40A306A39E37360C7A" ma:contentTypeVersion="4" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="15da9dc3ad285fe43873ecbef70e4065">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="37a59701-210d-47b6-ae01-fca6546d58ce" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="4b394c718fe06450b223b502efe64f27" ns2:_="">
     <xsd:import namespace="37a59701-210d-47b6-ae01-fca6546d58ce"/>
@@ -1179,15 +1193,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
@@ -1197,6 +1202,14 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{569F84B1-45EB-4542-821C-A957A49172A3}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{AAACEA31-FAFB-4C17-858C-8F27375FB9EA}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -1214,14 +1227,6 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{569F84B1-45EB-4542-821C-A957A49172A3}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0466E9FC-0FC4-4755-B69E-E404DE005AA0}">
   <ds:schemaRefs>

</xml_diff>